<commit_message>
BRD-04, BRD-05, BRD-06, BRD-07 and BRD-09 sources: a locked account is refused with the same message as a wrong password, the lock shows to the System Administrator; history column By of BRD-01 and BRD-03 names the user, with the role under it only for the users who may read the roles of others; FRS, sign-off workbooks and test plans that quote these texts rebuilt
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Drop-1_Transactional/BRD-04_Collections/BIBS_TestPlan_BRD-04_Collections_v1.0.xlsx
+++ b/docs/deliverables/out/Drop-1_Transactional/BRD-04_Collections/BIBS_TestPlan_BRD-04_Collections_v1.0.xlsx
@@ -8413,7 +8413,7 @@
       </c>
       <c r="H6" s="12" t="inlineStr">
         <is>
-          <t>Direct request outside the screens, signed in as the persona (test lead tool)</t>
+          <t>System function check outside the screens, signed in as the persona (test lead tool)</t>
         </is>
       </c>
       <c r="I6" s="12" t="inlineStr">
@@ -8716,8 +8716,8 @@
       </c>
       <c r="K10" s="12" t="inlineStr">
         <is>
-          <t>The third attempt locks the account; the correct password is refused until the System Administrator unlocks the user.
-Message "Account is locked. Contact your administrator." (AUTHENTICATION_FAILED).</t>
+          <t>The third attempt locks the account; the correct password is refused with the same message as a wrong password until the System Administrator unlocks the user in Administration &gt; Users, where the lock shows.
+Message "Invalid user name or password" (AUTHENTICATION_FAILED).</t>
         </is>
       </c>
       <c r="L10" s="12" t="inlineStr">
@@ -8992,7 +8992,7 @@
       </c>
       <c r="H14" s="12" t="inlineStr">
         <is>
-          <t>Direct request outside the screens, signed in as the persona (test lead tool)</t>
+          <t>System function check outside the screens, signed in as the persona (test lead tool)</t>
         </is>
       </c>
       <c r="I14" s="12" t="inlineStr">
@@ -9282,7 +9282,7 @@
       </c>
       <c r="H18" s="12" t="inlineStr">
         <is>
-          <t>Direct request outside the screens, signed in as the persona (test lead tool)</t>
+          <t>System function check outside the screens, signed in as the persona (test lead tool)</t>
         </is>
       </c>
       <c r="I18" s="12" t="inlineStr">
@@ -10923,7 +10923,7 @@
       </c>
       <c r="H41" s="12" t="inlineStr">
         <is>
-          <t>Direct request outside the screens, signed in as the persona (test lead tool)</t>
+          <t>System function check outside the screens, signed in as the persona (test lead tool)</t>
         </is>
       </c>
       <c r="I41" s="12" t="inlineStr">
@@ -12052,7 +12052,7 @@
       </c>
       <c r="I57" s="12" t="inlineStr">
         <is>
-          <t>The test lead makes the run fail on SIT (for example by stopping the database connection pool of the job).</t>
+          <t>The test lead makes the run fail on SIT (for example by stopping the connection of the job to its records).</t>
         </is>
       </c>
       <c r="J57" s="12" t="inlineStr">
@@ -12253,7 +12253,7 @@
       </c>
       <c r="H60" s="12" t="inlineStr">
         <is>
-          <t>Direct request outside the screens, signed in as the persona (test lead tool)</t>
+          <t>System function check outside the screens, signed in as the persona (test lead tool)</t>
         </is>
       </c>
       <c r="I60" s="12" t="inlineStr"/>
@@ -12465,7 +12465,7 @@
       </c>
       <c r="H63" s="12" t="inlineStr">
         <is>
-          <t>Direct request outside the screens, signed in as the persona (test lead tool)</t>
+          <t>System function check outside the screens, signed in as the persona (test lead tool)</t>
         </is>
       </c>
       <c r="I63" s="12" t="inlineStr">
@@ -13520,7 +13520,7 @@
       </c>
       <c r="H78" s="12" t="inlineStr">
         <is>
-          <t>Direct request outside the screens, signed in as the persona (test lead tool)</t>
+          <t>System function check outside the screens, signed in as the persona (test lead tool)</t>
         </is>
       </c>
       <c r="I78" s="12" t="inlineStr">
@@ -13665,7 +13665,7 @@
       </c>
       <c r="H80" s="12" t="inlineStr">
         <is>
-          <t>Direct request outside the screens, signed in as the persona (test lead tool)</t>
+          <t>System function check outside the screens, signed in as the persona (test lead tool)</t>
         </is>
       </c>
       <c r="I80" s="12" t="inlineStr">
@@ -13883,7 +13883,7 @@
       </c>
       <c r="H83" s="12" t="inlineStr">
         <is>
-          <t>Direct request outside the screens, signed in as the persona (test lead tool)</t>
+          <t>System function check outside the screens, signed in as the persona (test lead tool)</t>
         </is>
       </c>
       <c r="I83" s="12" t="inlineStr">
@@ -14240,7 +14240,7 @@
       </c>
       <c r="H88" s="12" t="inlineStr">
         <is>
-          <t>Direct request outside the screens, signed in as the persona (test lead tool)</t>
+          <t>System function check outside the screens, signed in as the persona (test lead tool)</t>
         </is>
       </c>
       <c r="I88" s="12" t="inlineStr">
@@ -14384,7 +14384,7 @@
       </c>
       <c r="H90" s="12" t="inlineStr">
         <is>
-          <t>Direct request outside the screens, signed in as the persona (test lead tool)</t>
+          <t>System function check outside the screens, signed in as the persona (test lead tool)</t>
         </is>
       </c>
       <c r="I90" s="12" t="inlineStr">
@@ -14456,7 +14456,7 @@
       </c>
       <c r="H91" s="12" t="inlineStr">
         <is>
-          <t>Direct request outside the screens, signed in as the persona (test lead tool)</t>
+          <t>System function check outside the screens, signed in as the persona (test lead tool)</t>
         </is>
       </c>
       <c r="I91" s="12" t="inlineStr">
@@ -14528,7 +14528,7 @@
       </c>
       <c r="H92" s="12" t="inlineStr">
         <is>
-          <t>Direct request outside the screens, signed in as the persona (test lead tool)</t>
+          <t>System function check outside the screens, signed in as the persona (test lead tool)</t>
         </is>
       </c>
       <c r="I92" s="12" t="inlineStr">
@@ -15176,7 +15176,7 @@
       </c>
       <c r="H101" s="12" t="inlineStr">
         <is>
-          <t>Direct request outside the screens, signed in as the persona (test lead tool)</t>
+          <t>System function check outside the screens, signed in as the persona (test lead tool)</t>
         </is>
       </c>
       <c r="I101" s="12" t="inlineStr">
@@ -15534,7 +15534,7 @@
       </c>
       <c r="H106" s="12" t="inlineStr">
         <is>
-          <t>Direct request outside the screens, signed in as the persona (test lead tool)</t>
+          <t>System function check outside the screens, signed in as the persona (test lead tool)</t>
         </is>
       </c>
       <c r="I106" s="12" t="inlineStr">
@@ -17406,7 +17406,7 @@
       </c>
       <c r="H132" s="12" t="inlineStr">
         <is>
-          <t>Direct request outside the screens, signed in as the persona (test lead tool)</t>
+          <t>System function check outside the screens, signed in as the persona (test lead tool)</t>
         </is>
       </c>
       <c r="I132" s="12" t="inlineStr">
@@ -18198,7 +18198,7 @@
       </c>
       <c r="H143" s="12" t="inlineStr">
         <is>
-          <t>Direct request outside the screens, signed in as the persona (test lead tool)</t>
+          <t>System function check outside the screens, signed in as the persona (test lead tool)</t>
         </is>
       </c>
       <c r="I143" s="12" t="inlineStr">
@@ -19255,7 +19255,7 @@
       </c>
       <c r="H158" s="12" t="inlineStr">
         <is>
-          <t>Direct request outside the screens, signed in as the persona (test lead tool)</t>
+          <t>System function check outside the screens, signed in as the persona (test lead tool)</t>
         </is>
       </c>
       <c r="I158" s="12" t="inlineStr">
@@ -20448,7 +20448,7 @@
       </c>
       <c r="H175" s="12" t="inlineStr">
         <is>
-          <t>Direct request outside the screens, signed in as the persona (test lead tool)</t>
+          <t>System function check outside the screens, signed in as the persona (test lead tool)</t>
         </is>
       </c>
       <c r="I175" s="12" t="inlineStr">
@@ -21871,7 +21871,7 @@
       </c>
       <c r="H195" s="12" t="inlineStr">
         <is>
-          <t>Direct request outside the screens, signed in as the persona (test lead tool)</t>
+          <t>System function check outside the screens, signed in as the persona (test lead tool)</t>
         </is>
       </c>
       <c r="I195" s="12" t="inlineStr">
@@ -22159,7 +22159,7 @@
       </c>
       <c r="H199" s="12" t="inlineStr">
         <is>
-          <t>Direct request outside the screens, signed in as the persona (test lead tool)</t>
+          <t>System function check outside the screens, signed in as the persona (test lead tool)</t>
         </is>
       </c>
       <c r="I199" s="12" t="inlineStr">
@@ -23166,7 +23166,7 @@
       </c>
       <c r="H213" s="12" t="inlineStr">
         <is>
-          <t>Direct request outside the screens, signed in as the persona (test lead tool)</t>
+          <t>System function check outside the screens, signed in as the persona (test lead tool)</t>
         </is>
       </c>
       <c r="I213" s="12" t="inlineStr">
@@ -23439,7 +23439,7 @@
       </c>
       <c r="H217" s="12" t="inlineStr">
         <is>
-          <t>Direct request outside the screens, signed in as the persona (test lead tool)</t>
+          <t>System function check outside the screens, signed in as the persona (test lead tool)</t>
         </is>
       </c>
       <c r="I217" s="12" t="inlineStr"/>

</xml_diff>